<commit_message>
update for revision -1st round
</commit_message>
<xml_diff>
--- a/Summarized_Results.xlsx
+++ b/Summarized_Results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\25244\Desktop\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B3F03B-F1B3-4399-A1E2-541CE7CA8FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E75F6FD1-F29A-4808-8479-6E1D8D3C2CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11100" yWindow="1540" windowWidth="12470" windowHeight="11130" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SE Tasks" sheetId="1" r:id="rId1"/>
@@ -49,18 +49,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Reusability (1)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Fault tolerance (21)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Faultlessness (13)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Confidentiality (9)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -77,14 +65,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Reliability (34)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Compatibility (10)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Security (10)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -97,62 +77,18 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Self-Reflection (34)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Retrieval-Augmented Generation (10)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Debate-Based Cooperation (4)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Layered-Based Cooperation (4)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Agent Evaluator (3)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Multi-Path Plan Generator (3)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Incremental Model Querying (3)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Hierarchical Coordination (3)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Voting-Based Cooperation (3)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Code Generation (45)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Fault Localization (9)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Program Repair (8)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Software Testing (6)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>End-to-End Software Maintenance (8)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Code Translation (1)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -161,71 +97,203 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Improving the Efficiency of Generating Software Artifacts (23)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Optimizing Software Resource Management (27)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>End-to-End Software Development (7)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Code Review (6)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Functional Correctness (86)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Functional Appropriateness (11)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Performance Efficiency (48)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Resource Utilization (27)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Analysability (4)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Flexibility (24)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Adaptability (16)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Scalability (12)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Interoperability (8)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Cross-Reflection (12)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Single-Path Plan Generator (5)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Prompt/Response Optimiser (4)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Improving the Quality of Generated Code (42)</t>
+    <t>Human-Reflection (5)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Co-Existence (7)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Release Management (1)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Capacity (11)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ensuring Software Security (3)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Code Generation (49)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>End-to-End Software Development (11)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fault Localization (10)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>End-to-End Software Maintenance (9)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Software Testing (7)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Requirements Engineering (4)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Functional Suitability (101)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Functional Correctness (97)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Functional Completeness (26)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Functional Appropriateness (12)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Performance Efficiency (51)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Resource Utilization (29)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Time Behavior (29)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Maintainability (55)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Modularity (53)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Analysability (5)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reusability (2)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reliability (40)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fault tolerance (24)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Faultlessness (16)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Flexibility (30)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Adaptability (21)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scalability (13)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Compatibility (12)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Interoperability (10)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Role-Based Cooperation (49)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Self-Reflection (36)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tool-Agent Registry (16)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cross-Reflection (14)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Retrieval-Augmented Generation (12)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Incremental Model Querying (10)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Agent Adapter (8)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Single-Path Plan Generator (7)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Debate-Based Cooperation (5)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hierarchical Coordination (5)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Agent Evaluator (4)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Multi-Path Plan Generator (4)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Improving the Quality of Generated Code (51)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Simulating Human Processes of Solving SE Tasks (31)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Optimizing Software Resource Management (29)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Improving the Efficiency of Generating Software Artifacts (25)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reducing the Difficulty of Task Resolution (25)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Improving the Adaptability of Agent Systems (20)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -252,76 +320,8 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>12)</t>
+      <t>14)</t>
     </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Requirements Engineering (3)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Functional Completeness (24)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Functional Suitability (89)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Modularity (46)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Maintainability (47)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Role-Based Cooperation (44)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Simulating Human Processes of Solving SE Tasks (28)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Agent Adapter (6)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Human-Reflection (5)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Co-Existence (7)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Release Management (1)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Improving the Adaptability of Agent Systems (18)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Time Behavior (27)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Capacity (11)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Reducing the Difficulty of Task Resolution (20)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ensuring Software Security (3)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Tool-Agent Registry (14)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -743,7 +743,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -751,7 +751,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -759,7 +759,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -767,7 +767,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -775,7 +775,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -783,7 +783,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -791,7 +791,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -799,7 +799,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -807,7 +807,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -815,7 +815,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -850,10 +850,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
@@ -861,7 +861,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="C3" s="12"/>
     </row>
@@ -870,7 +870,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C4" s="12"/>
     </row>
@@ -879,10 +879,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
@@ -890,7 +890,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="C6" s="11"/>
     </row>
@@ -899,7 +899,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="C7" s="11"/>
     </row>
@@ -908,10 +908,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
@@ -919,7 +919,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C9" s="11"/>
     </row>
@@ -928,7 +928,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C10" s="11"/>
     </row>
@@ -937,10 +937,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>6</v>
+        <v>42</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
@@ -948,7 +948,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="C12" s="11"/>
     </row>
@@ -957,10 +957,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
@@ -968,7 +968,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C14" s="11"/>
     </row>
@@ -977,10 +977,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
@@ -988,7 +988,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="C16" s="11"/>
     </row>
@@ -997,10 +997,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
@@ -1008,7 +1008,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C18" s="11"/>
     </row>
@@ -1017,10 +1017,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>10</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
@@ -1028,7 +1028,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C20" s="11"/>
     </row>
@@ -1048,8 +1048,8 @@
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="C11:C12"/>
     <mergeCell ref="C2:C4"/>
+    <mergeCell ref="C8:C10"/>
     <mergeCell ref="C5:C7"/>
-    <mergeCell ref="C8:C10"/>
     <mergeCell ref="C13:C14"/>
     <mergeCell ref="C15:C16"/>
   </mergeCells>
@@ -1071,7 +1071,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1079,7 +1079,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1087,7 +1087,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1095,7 +1095,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1103,7 +1103,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1111,7 +1111,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1119,7 +1119,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1127,7 +1127,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1135,7 +1135,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1143,7 +1143,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1151,7 +1151,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>19</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1159,7 +1159,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1167,7 +1167,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1175,7 +1175,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1183,7 +1183,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1191,7 +1191,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1199,7 +1199,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1221,7 +1221,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1229,7 +1229,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1237,7 +1237,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1245,7 +1245,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1253,7 +1253,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1269,7 +1269,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1277,7 +1277,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1285,7 +1285,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>66</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">

</xml_diff>